<commit_message>
Add broadly_expressed_detectable tier + drug targets
Resolves the BMAp/RE/DG zero-pick problem without lowering the gold
standard. Genes that pct>=50%, log2>=4, spec>=-2 are now surfaced as
'broadly_expressed_detectable' tier 2 in combined_GPCRs_for_probe.
Original tier 1 (specificity_log2 > 0) remains unchanged.

New: v3/inputs/gpcr_drug_targets.csv (39 GPCRs) drives a GPCR_Drug_Targets
workbook sheet and a per-cell-type existing_drugs_for_picks column.
Inline drug info is also embedded in combined_GPCRs_for_probe entries.

Configurable via three new keys in project_config.yaml:
  broad_min_pct_expr (50), broad_min_mean_log2_expr (4.0),
  broad_min_specificity_log2 (-2.0).

Result: BMAp/RE/DG/LM/CA-DG anchors that previously had 0 picks now
each surface 2-4 broadly-detectable candidates with FDA/clinical drug
context for downstream pharmacology lookup.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/FINAL_decision_table_combined.xlsx
+++ b/outputs/FINAL_decision_table_combined.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +66,11 @@
         <fgColor rgb="00F4B084"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C9A0DC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -85,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -103,6 +108,9 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,7 +542,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  combined_GPCRs_for_probe    = UNION of paper + Allen, each gene tagged: paper+allen_keep | allen_only_keep | paper_only_allen_downgrade</t>
+          <t xml:space="preserve">  combined_GPCRs_for_probe    = UNION of paper + Allen, tagged paper+allen_keep | allen_only_keep | paper+allen_broadly_detectable | allen_only_broadly_detectable | paper_only_allen_downgrade</t>
         </is>
       </c>
     </row>
@@ -544,7 +552,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  combined_evidence_summary   = compact summary: which genes match, which are paper-only with downgrade reason, which are Allen-found-new</t>
+          <t xml:space="preserve">  combined_evidence_summary   = compact summary of which genes were kept and why</t>
         </is>
       </c>
     </row>
@@ -554,7 +562,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Recommended order list = combined_GPCRs_for_probe (use paper+allen_keep first; then allen_only_keep; then paper_only with FISH validation)</t>
+          <t xml:space="preserve">  n_GPCRs_keep                = count of cell-type-specific genes (Allen keep tier)</t>
         </is>
       </c>
     </row>
@@ -563,6 +571,36 @@
         <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  n_broadly_detectable        = count of broadly-expressed but reliably-detectable genes (use only if region/spatial constrained)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  existing_drugs_for_picks    = FDA-approved + clinical/research drugs targeting genes in the union list</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Recommended order = combined_GPCRs_for_probe (paper+allen_keep &gt; allen_only_keep &gt; broadly_detectable &gt; paper_only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Generated by D04_make_focused_decision_table.py from v3/outputs/Final_Probe_Panel_v7_modular.xlsx (Final_Summary sheet)</t>
         </is>
@@ -579,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -590,9 +628,12 @@
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="110" customWidth="1" min="9" max="9"/>
+    <col width="130" customWidth="1" min="9" max="9"/>
     <col width="90" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="90" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -648,925 +689,1138 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
+          <t>n_GPCRs_keep</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>n_broadly_detectable</t>
+        </is>
+      </c>
+      <c r="M1" s="7" t="inlineStr">
+        <is>
+          <t>existing_drugs_for_picks</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
           <t>warning</t>
         </is>
       </c>
     </row>
     <row r="2" ht="110" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>D1/direct-pathway SPN</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>061 STR D1 Gaba</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" s="8" t="n">
         <v>16660</v>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>Drd1, Isl1, Pdyn, Tac1</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>Adora2a, Drd2, Penk</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Chrm4, Cnr1, Drd1, Gabbr1, Gpr88, Grm1, Grm5, Htr1b, Oprd1, Oprm1</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>Drd1(spec=0.44, log2=8.77, pct=100%, status=keep); Grm1(spec=0.22, log2=8.99, pct=99%, status=keep); Htr1b(spec=0.15, log2=6.50, pct=93%, status=keep); Chrm4(spec=0.00, log2=0.27, pct=6%, status=candidate_to_validate)</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
-        <is>
-          <t>Drd1[paper+allen_keep, spec=+0.44, log2=8.77, pct=100%]; Grm1[paper+allen_keep, spec=+0.22, log2=8.99, pct=99%]; Htr1b[paper+allen_keep, spec=+0.15, log2=6.50, pct=93%]; Chrm4[paper+allen_keep, spec=+0.00, log2=0.27, pct=6%]; Cnr1[paper_only_allen_downgrade, spec=-1.92, log2=7.76, pct=93%]; Gabbr1[paper_only_allen_downgrade, spec=-0.59, log2=8.59, pct=100%]; Gpr88[paper_only_allen_downgrade, spec=-0.76, log2=10.17, pct=100%]; Grm5[paper_only_allen_downgrade, spec=-0.02, log2=11.36, pct=100%]; Oprd1[paper_only_allen_downgrade, spec=-5.76, log2=0.13, pct=2%]; Oprm1[paper_only_allen_downgrade, spec=-5.12, log2=2.83, pct=44%]</t>
-        </is>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
-        <is>
-          <t>both: Drd1, Grm1, Htr1b, Chrm4 | paper_only: Cnr1(downgrade,spec=-1.92,log2=7.76); Gabbr1(downgrade,spec=-0.59,log2=8.59); Gpr88(downgrade,spec=-0.76,log2=10.17); Grm5(downgrade,spec=-0.02,log2=11.36); Oprd1(downgrade,spec=-5.76,log2=0.13); Oprm1(downgrade,spec=-5.12,log2=2.83)</t>
-        </is>
-      </c>
-      <c r="K2" s="7" t="inlineStr"/>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Drd1[paper+allen_keep, spec=+0.44, log2=8.77, pct=100%; drugs: Apomorphine (mixed); Pergolide (partial)]; Grm1[paper+allen_keep, spec=+0.22, log2=8.99, pct=99%; drugs: research_only_or_none]; Htr1b[paper+allen_keep, spec=+0.15, log2=6.50, pct=93%; drugs: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan]; Chrm4[paper+allen_keep, spec=+0.00, log2=0.27, pct=6%; drugs: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia)]; Cnr1[paper+allen_broadly_detectable, spec=-1.92, log2=7.76, pct=93%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Gabbr1[paper+allen_broadly_detectable, spec=-0.59, log2=8.59, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gpr88[paper+allen_broadly_detectable, spec=-0.76, log2=10.17, pct=100%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-0.02, log2=11.36, pct=100%; drugs: research_only_or_none]; Htr2c[allen_only_broadly_detectable, spec=-0.75, log2=7.00, pct=94%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Oprd1[paper_only_allen_downgrade, spec=-5.76, log2=0.13, pct=2%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-5.12, log2=2.83, pct=44%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Drd1, Grm1, Htr1b, Chrm4 | paper+broadly_detectable: Cnr1, Gabbr1, Gpr88, Grm5 | allen_only_broadly_detectable: Htr2c | paper_only: Oprd1(downgrade,spec=-5.76,log2=0.13); Oprm1(downgrade,spec=-5.12,log2=2.83)</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
+        <is>
+          <t>Drd1 | FDA: Apomorphine (mixed); Pergolide (partial) | clinical/research: SKF-81297; SKF-38393 (research agonists); SCH-23390 (antagonist) | indication: Parkinson disease; addiction research || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Htr1b | FDA: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan | indication: migraine (acute attack) || Chrm4 | FDA: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia) | indication: schizophrenia || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gpr88 | clinical/research: RTI-13951-33 (research agonist) | indication: obsessive-compulsive disorder; addiction (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia</t>
+        </is>
+      </c>
+      <c r="N2" s="8" t="inlineStr"/>
     </row>
     <row r="3" ht="110" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>D1/direct-pathway SPN</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>063 STR D1 Sema5a Gaba</t>
         </is>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="8" t="n">
         <v>780</v>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Drd1, Isl1, Pdyn, Tac1</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Adora2a, Drd2, Penk</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Chrm4, Cnr1, Drd1, Gabbr1, Gpr88, Grm1, Grm5, Htr1b, Oprd1, Oprm1</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr"/>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>Chrm4[paper_only_allen_downgrade, spec=-0.00, log2=0.27, pct=6%]; Cnr1[paper_only_allen_downgrade, spec=-2.88, log2=6.79, pct=85%]; Drd1[paper_only_allen_downgrade, spec=-0.44, log2=8.33, pct=99%]; Gabbr1[paper_only_allen_downgrade, spec=-0.65, log2=8.53, pct=100%]; Gpr88[paper_only_allen_downgrade, spec=-0.22, log2=10.70, pct=100%]; Grm1[paper_only_allen_downgrade, spec=-4.63, log2=4.36, pct=68%]; Grm5[paper_only_allen_downgrade, spec=-1.04, log2=10.34, pct=100%]; Htr1b[paper_only_allen_downgrade, spec=-3.19, log2=3.31, pct=55%]; Oprd1[paper_only_allen_downgrade, spec=-5.21, log2=0.68, pct=13%]; Oprm1[paper_only_allen_downgrade, spec=-3.98, log2=3.97, pct=61%]</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Chrm4(downgrade,spec=-0.00,log2=0.27); Cnr1(downgrade,spec=-2.88,log2=6.79); Drd1(downgrade,spec=-0.44,log2=8.33); Gabbr1(downgrade,spec=-0.65,log2=8.53); Gpr88(downgrade,spec=-0.22,log2=10.70); Grm1(downgrade,spec=-4.63,log2=4.36); Grm5(downgrade,spec=-1.04,log2=10.34); Htr1b(downgrade,spec=-3.19,log2=3.31); Oprd1(downgrade,spec=-5.21,log2=0.68); Oprm1(downgrade,spec=-3.98,log2=3.97)</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H3" s="8" t="inlineStr"/>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Drd1[paper+allen_broadly_detectable, spec=-0.44, log2=8.33, pct=99%; drugs: Apomorphine (mixed); Pergolide (partial)]; Gabbr1[paper+allen_broadly_detectable, spec=-0.65, log2=8.53, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gpr88[paper+allen_broadly_detectable, spec=-0.22, log2=10.70, pct=100%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-1.04, log2=10.34, pct=100%; drugs: research_only_or_none]; Chrm4[paper_only_allen_downgrade, spec=-0.00, log2=0.27, pct=6%; drugs: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia)]; Cnr1[paper_only_allen_downgrade, spec=-2.88, log2=6.79, pct=85%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Grm1[paper_only_allen_downgrade, spec=-4.63, log2=4.36, pct=68%; drugs: research_only_or_none]; Htr1b[paper_only_allen_downgrade, spec=-3.19, log2=3.31, pct=55%; drugs: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan]; Oprd1[paper_only_allen_downgrade, spec=-5.21, log2=0.68, pct=13%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-3.98, log2=3.97, pct=61%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Drd1, Gabbr1, Gpr88, Grm5 | paper_only: Chrm4(downgrade,spec=-0.00,log2=0.27); Cnr1(downgrade,spec=-2.88,log2=6.79); Grm1(downgrade,spec=-4.63,log2=4.36); Htr1b(downgrade,spec=-3.19,log2=3.31); Oprd1(downgrade,spec=-5.21,log2=0.68); Oprm1(downgrade,spec=-3.98,log2=3.97)</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Drd1 | FDA: Apomorphine (mixed); Pergolide (partial) | clinical/research: SKF-81297; SKF-38393 (research agonists); SCH-23390 (antagonist) | indication: Parkinson disease; addiction research || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gpr88 | clinical/research: RTI-13951-33 (research agonist) | indication: obsessive-compulsive disorder; addiction (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Chrm4 | FDA: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia) | indication: schizophrenia || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Htr1b | FDA: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan | indication: migraine (acute attack) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 4 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>
     <row r="4" ht="110" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>D2/indirect-pathway SPN</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>062 STR D2 Gaba</t>
         </is>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="8" t="n">
         <v>18139</v>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Adora2a, Drd2, Gpr52, Gpr6, Penk, Sp9</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="8" t="inlineStr">
         <is>
           <t>Drd1, Tac1</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Adora2a, Chrm4, Cnr1, Drd2, Gpr52, Gpr6, Gpr88, Grm1, Grm5, Oprd1</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>Grm5(spec=0.02, log2=11.38, pct=100%, status=keep); Gpr88(spec=0.22, log2=10.92, pct=100%, status=keep); Drd2(spec=0.24, log2=9.26, pct=99%, status=keep); Adora2a(spec=4.32, log2=9.20, pct=99%, status=keep); Gpr6(spec=5.74, log2=6.45, pct=93%, status=keep); Gpr52(spec=2.26, log2=2.78, pct=50%, status=keep)</t>
         </is>
       </c>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>Grm5[paper+allen_keep, spec=+0.02, log2=11.38, pct=100%]; Gpr88[paper+allen_keep, spec=+0.22, log2=10.92, pct=100%]; Drd2[paper+allen_keep, spec=+0.24, log2=9.26, pct=99%]; Adora2a[paper+allen_keep, spec=+4.32, log2=9.20, pct=99%]; Gpr6[paper+allen_keep, spec=+5.74, log2=6.45, pct=93%]; Gpr52[paper+allen_keep, spec=+2.26, log2=2.78, pct=50%]; Chrm4[paper_only_allen_downgrade, spec=-0.27, log2=0.01, pct=0%]; Cnr1[paper_only_allen_downgrade, spec=-2.40, log2=7.28, pct=88%]; Grm1[paper_only_allen_downgrade, spec=-0.22, log2=8.77, pct=98%]; Oprd1[paper_only_allen_downgrade, spec=-2.02, log2=3.86, pct=64%]</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>both: Grm5, Gpr88, Drd2, Adora2a, Gpr6, Gpr52 | paper_only: Chrm4(downgrade,spec=-0.27,log2=0.01); Cnr1(downgrade,spec=-2.40,log2=7.28); Grm1(downgrade,spec=-0.22,log2=8.77); Oprd1(downgrade,spec=-2.02,log2=3.86)</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Grm5[paper+allen_keep, spec=+0.02, log2=11.38, pct=100%; drugs: research_only_or_none]; Gpr88[paper+allen_keep, spec=+0.22, log2=10.92, pct=100%; drugs: research_only_or_none]; Drd2[paper+allen_keep, spec=+0.24, log2=9.26, pct=99%; drugs: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect)]; Adora2a[paper+allen_keep, spec=+4.32, log2=9.20, pct=99%; drugs: Istradefylline (Nourianz; FDA 2019)]; Gpr6[paper+allen_keep, spec=+5.74, log2=6.45, pct=93%; drugs: research_only_or_none]; Gpr52[paper+allen_keep, spec=+2.26, log2=2.78, pct=50%; drugs: research_only_or_none]; Grm1[paper+allen_broadly_detectable, spec=-0.22, log2=8.77, pct=98%; drugs: research_only_or_none]; Gabbr1[allen_only_broadly_detectable, spec=-0.69, log2=8.49, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Htr1b[allen_only_broadly_detectable, spec=-0.15, log2=6.35, pct=90%; drugs: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan]; Htr2c[allen_only_broadly_detectable, spec=-0.41, log2=7.34, pct=94%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Chrm4[paper_only_allen_downgrade, spec=-0.27, log2=0.01, pct=0%; drugs: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia)]; Cnr1[paper_only_allen_downgrade, spec=-2.40, log2=7.28, pct=88%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Oprd1[paper_only_allen_downgrade, spec=-2.02, log2=3.86, pct=64%; drugs: research_only_or_none]</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Grm5, Gpr88, Drd2, Adora2a, Gpr6, Gpr52 | paper+broadly_detectable: Grm1 | allen_only_broadly_detectable: Gabbr1, Htr1b, Htr2c | paper_only: Chrm4(downgrade,spec=-0.27,log2=0.01); Cnr1(downgrade,spec=-2.40,log2=7.28); Oprd1(downgrade,spec=-2.02,log2=3.86)</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M4" s="8" t="inlineStr">
+        <is>
+          <t>Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Gpr88 | clinical/research: RTI-13951-33 (research agonist) | indication: obsessive-compulsive disorder; addiction (preclinical) || Drd2 | FDA: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect) | clinical/research: many | indication: schizophrenia; bipolar; Parkinson disease; hyperprolactinemia || Adora2a | FDA: Istradefylline (Nourianz; FDA 2019) | clinical/research: Caffeine (non-selective); Preladenant (discontinued); Tozadenant | indication: Parkinson disease (adjunct to levodopa) || Gpr6 | clinical/research: research antagonists for Parkinson disease | indication: Parkinson research (preclinical) || Gpr52 | clinical/research: FTBMT (research agonist for Huntington); experimental Lundbeck/Mitsubishi compounds | indication: Huntington disease; schizophrenia (preclinical) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Htr1b | FDA: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan | indication: migraine (acute attack) || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Chrm4 | FDA: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia) | indication: schizophrenia || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical)</t>
+        </is>
+      </c>
+      <c r="N4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="110" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>CP</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Cholinergic interneuron</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>058 PAL-STR Gaba-Chol</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Chat, Lhx8, Slc18a3, Slc5a7</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Drd1, Drd2</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Adora2a, Chrm2, Chrm4, Cnr1, Drd2, Gabbr1, Oprm1, Tacr1</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Gabbr1(spec=0.59, log2=9.18, pct=100%, status=keep); Chrm2(spec=0.32, log2=8.97, pct=100%, status=keep); Oprm1(spec=1.08, log2=7.95, pct=100%, status=keep); Tacr3(spec=3.71, log2=7.12, pct=93%, status=keep); Oprd1(spec=2.02, log2=5.88, pct=97%, status=keep); Hcrtr2(spec=3.07, log2=4.37, pct=77%, status=keep); Crhr1(spec=0.14, log2=3.07, pct=67%, status=keep)</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
-        <is>
-          <t>Gabbr1[paper+allen_keep, spec=+0.59, log2=9.18, pct=100%]; Chrm2[paper+allen_keep, spec=+0.32, log2=8.97, pct=100%]; Oprm1[paper+allen_keep, spec=+1.08, log2=7.95, pct=100%]; Tacr3[allen_only_keep, spec=+3.71, log2=7.12, pct=93%]; Oprd1[allen_only_keep, spec=+2.02, log2=5.88, pct=97%]; Hcrtr2[allen_only_keep, spec=+3.07, log2=4.37, pct=77%]; Crhr1[allen_only_keep, spec=+0.14, log2=3.07, pct=67%]; Adora2a[paper_only_allen_downgrade, spec=-7.84, log2=1.36, pct=33%]; Chrm4[paper_only_allen_downgrade, spec=-0.27, log2=0.00, pct=0%]; Cnr1[paper_only_allen_downgrade, spec=-7.31, log2=2.37, pct=50%]; Drd2[paper_only_allen_downgrade, spec=-0.24, log2=9.02, pct=100%]; Tacr1[paper_only_allen_downgrade, spec=-0.52, log2=9.99, pct=100%]</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>both: Gabbr1, Chrm2, Oprm1 | paper_only: Adora2a(downgrade,spec=-7.84,log2=1.36); Chrm4(downgrade,spec=-0.27,log2=0.00); Cnr1(downgrade,spec=-7.31,log2=2.37); Drd2(downgrade,spec=-0.24,log2=9.02); Tacr1(downgrade,spec=-0.52,log2=9.99) | allen_only_keep: Tacr3, Oprd1, Hcrtr2, Crhr1</t>
-        </is>
-      </c>
-      <c r="K5" s="7" t="inlineStr"/>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_keep, spec=+0.59, log2=9.18, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Chrm2[paper+allen_keep, spec=+0.32, log2=8.97, pct=100%; drugs: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic)]; Oprm1[paper+allen_keep, spec=+1.08, log2=7.95, pct=100%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Tacr3[allen_only_keep, spec=+3.71, log2=7.12, pct=93%; drugs: Fezolinetant (Veozah; FDA 2023); Elinzanetant (in trials)]; Oprd1[allen_only_keep, spec=+2.02, log2=5.88, pct=97%; drugs: research_only_or_none]; Hcrtr2[allen_only_keep, spec=+3.07, log2=4.37, pct=77%; drugs: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2]; Crhr1[allen_only_keep, spec=+0.14, log2=3.07, pct=67%; drugs: research_only_or_none]; Drd2[paper+allen_broadly_detectable, spec=-0.24, log2=9.02, pct=100%; drugs: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect)]; Tacr1[paper+allen_broadly_detectable, spec=-0.52, log2=9.99, pct=100%; drugs: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet)]; Adcyap1r1[allen_only_broadly_detectable, spec=-1.85, log2=4.69, pct=87%; drugs: research_only_or_none]; Htr2c[allen_only_broadly_detectable, spec=-1.75, log2=6.00, pct=93%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Adora2a[paper_only_allen_downgrade, spec=-7.84, log2=1.36, pct=33%; drugs: Istradefylline (Nourianz; FDA 2019)]; Chrm4[paper_only_allen_downgrade, spec=-0.27, log2=0.00, pct=0%; drugs: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia)]; Cnr1[paper_only_allen_downgrade, spec=-7.31, log2=2.37, pct=50%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Gabbr1, Chrm2, Oprm1 | allen_only_keep: Tacr3, Oprd1, Hcrtr2, Crhr1 | paper+broadly_detectable: Drd2, Tacr1 | allen_only_broadly_detectable: Adcyap1r1, Htr2c | paper_only: Adora2a(downgrade,spec=-7.84,log2=1.36); Chrm4(downgrade,spec=-0.27,log2=0.00); Cnr1(downgrade,spec=-7.31,log2=2.37)</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Chrm2 | FDA: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic) | clinical/research: Methoctramine (research) | indication: Alzheimer disease; overactive bladder || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Tacr3 | FDA: Fezolinetant (Veozah; FDA 2023); Elinzanetant (in trials) | clinical/research: MK-3207 | indication: vasomotor symptoms (menopausal hot flashes) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Hcrtr2 | FDA: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2 | clinical/research: JNJ-42847922 (selective OX2R) | indication: insomnia || Crhr1 | clinical/research: Verucerfont; Pexacerfont; Antalarmin; Emicerfont (depression/PTSD trials mostly failed) | indication: PTSD; major depression; alcohol use disorder (mostly failed) || Drd2 | FDA: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect) | clinical/research: many | indication: schizophrenia; bipolar; Parkinson disease; hyperprolactinemia || Tacr1 | FDA: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet) | indication: chemotherapy-induced nausea/vomiting (CINV); postoperative nausea || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Adora2a | FDA: Istradefylline (Nourianz; FDA 2019) | clinical/research: Caffeine (non-selective); Preladenant (discontinued); Tozadenant | indication: Parkinson disease (adjunct to levodopa) || Chrm4 | FDA: Xanomeline (in KarXT/Cobenfy; FDA Sept 2024 for schizophrenia) | indication: schizophrenia || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD)</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr"/>
     </row>
     <row r="6" ht="110" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>BMAp</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Posterior BMA glutamatergic VGLUT1-like</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>012 MEA Slc17a7 Glut</t>
         </is>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="8" t="n">
         <v>3984</v>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>C1ql2, Cartpt, Dcn, Gpr101, Meis2, Slc17a7</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>Gad1, Gad2, Slc32a1</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Cckbr, Cnr1, Crhr1, Gabbr1, Gabbr2, Gpr101, Grm5, Htr2c, Npy1r, Oprd1, Oprm1, Sstr2, Tacr1</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr"/>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>Cckbr[paper_only_allen_downgrade, spec=-3.12, log2=3.31, pct=58%]; Cnr1[paper_only_allen_downgrade, spec=-7.56, log2=3.94, pct=65%]; Crhr1[paper_only_allen_downgrade, spec=-1.34, log2=2.20, pct=41%]; Gabbr1[paper_only_allen_downgrade, spec=-0.71, log2=8.18, pct=100%]; Gabbr2[paper_only_allen_downgrade, spec=-1.23, log2=8.68, pct=100%]; Gpr101[paper_only_allen_downgrade, spec=-4.05, log2=2.94, pct=44%]; Grm5[paper_only_allen_downgrade, spec=-0.93, log2=10.54, pct=100%]; Htr2c[paper_only_allen_downgrade, spec=-5.59, log2=3.99, pct=59%]; Npy1r[paper_only_allen_downgrade, spec=-3.69, log2=3.64, pct=62%]; Oprd1[paper_only_allen_downgrade, spec=-4.98, log2=0.56, pct=11%]; Oprm1[paper_only_allen_downgrade, spec=-3.70, log2=3.70, pct=61%]; Sstr2[paper_only_allen_downgrade, spec=-2.64, log2=2.11, pct=40%]; Tacr1[paper_only_allen_downgrade, spec=-3.02, log2=3.94, pct=62%]</t>
-        </is>
-      </c>
-      <c r="J6" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Cckbr(downgrade,spec=-3.12,log2=3.31); Cnr1(downgrade,spec=-7.56,log2=3.94); Crhr1(downgrade,spec=-1.34,log2=2.20); Gabbr1(downgrade,spec=-0.71,log2=8.18); Gabbr2(downgrade,spec=-1.23,log2=8.68); Gpr101(downgrade,spec=-4.05,log2=2.94); Grm5(downgrade,spec=-0.93,log2=10.54); Htr2c(downgrade,spec=-5.59,log2=3.99); Npy1r(downgrade,spec=-3.69,log2=3.64); Oprd1(downgrade,spec=-4.98,log2=0.56); Oprm1(downgrade,spec=-3.70,log2=3.70); Sstr2(downgrade,spec=-2.64,log2=2.11); Tacr1(downgrade,spec=-3.02,log2=3.94)</t>
-        </is>
-      </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H6" s="8" t="inlineStr"/>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_broadly_detectable, spec=-0.71, log2=8.18, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.23, log2=8.68, pct=100%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm5[paper+allen_broadly_detectable, spec=-0.93, log2=10.54, pct=100%; drugs: research_only_or_none]; Npy2r[allen_only_broadly_detectable, spec=-0.62, log2=5.07, pct=76%; drugs: research_only_or_none]; Cckbr[paper_only_allen_downgrade, spec=-3.12, log2=3.31, pct=58%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-7.56, log2=3.94, pct=65%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Crhr1[paper_only_allen_downgrade, spec=-1.34, log2=2.20, pct=41%; drugs: research_only_or_none]; Gpr101[paper_only_allen_downgrade, spec=-4.05, log2=2.94, pct=44%; drugs: research_only_or_none]; Htr2c[paper_only_allen_downgrade, spec=-5.59, log2=3.99, pct=59%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Npy1r[paper_only_allen_downgrade, spec=-3.69, log2=3.64, pct=62%; drugs: research_only_or_none]; Oprd1[paper_only_allen_downgrade, spec=-4.98, log2=0.56, pct=11%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-3.70, log2=3.70, pct=61%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Sstr2[paper_only_allen_downgrade, spec=-2.64, log2=2.11, pct=40%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]; Tacr1[paper_only_allen_downgrade, spec=-3.02, log2=3.94, pct=62%; drugs: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet)]</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Gabbr1, Gabbr2, Grm5 | allen_only_broadly_detectable: Npy2r | paper_only: Cckbr(downgrade,spec=-3.12,log2=3.31); Cnr1(downgrade,spec=-7.56,log2=3.94); Crhr1(downgrade,spec=-1.34,log2=2.20); Gpr101(downgrade,spec=-4.05,log2=2.94); Htr2c(downgrade,spec=-5.59,log2=3.99); Npy1r(downgrade,spec=-3.69,log2=3.64); Oprd1(downgrade,spec=-4.98,log2=0.56); Oprm1(downgrade,spec=-3.70,log2=3.70); Sstr2(downgrade,spec=-2.64,log2=2.11); Tacr1(downgrade,spec=-3.02,log2=3.94)</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Npy2r | clinical/research: BIIE-0246 (research antagonist) | indication: food intake; anxiety (preclinical) || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Crhr1 | clinical/research: Verucerfont; Pexacerfont; Antalarmin; Emicerfont (depression/PTSD trials mostly failed) | indication: PTSD; major depression; alcohol use disorder (mostly failed) || Gpr101 | clinical/research: research only (orphan) | indication: X-LAG / X-linked acrogigantism research || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Npy1r | clinical/research: BIBP-3226 (research antagonist) | indication: obesity; pain (preclinical) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease || Tacr1 | FDA: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet) | indication: chemotherapy-induced nausea/vomiting (CINV); postoperative nausea</t>
+        </is>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 4 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>
     <row r="7" ht="110" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>BMAp</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Posterior BMA glutamatergic VGLUT1-like</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>113 MEA-COA-BMA Ccdc42 Glut</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="8" t="n">
         <v>9654</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>C1ql2, Cartpt, Dcn, Gpr101, Meis2, Slc17a7</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>Gad1, Gad2, Slc32a1</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Cckbr, Cnr1, Crhr1, Gabbr1, Gabbr2, Gpr101, Grm5, Htr2c, Npy1r, Oprd1, Oprm1, Sstr2, Tacr1</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Cckbr[paper_only_allen_downgrade, spec=-3.22, log2=3.22, pct=56%]; Cnr1[paper_only_allen_downgrade, spec=-10.94, log2=0.57, pct=10%]; Crhr1[paper_only_allen_downgrade, spec=-1.36, log2=2.19, pct=39%]; Gabbr1[paper_only_allen_downgrade, spec=-0.61, log2=8.28, pct=99%]; Gabbr2[paper_only_allen_downgrade, spec=-1.53, log2=8.38, pct=99%]; Gpr101[paper_only_allen_downgrade, spec=-3.42, log2=3.57, pct=57%]; Grm5[paper_only_allen_downgrade, spec=-1.12, log2=10.36, pct=100%]; Htr2c[paper_only_allen_downgrade, spec=-2.20, log2=7.38, pct=87%]; Npy1r[paper_only_allen_downgrade, spec=-3.62, log2=3.71, pct=62%]; Oprd1[paper_only_allen_downgrade, spec=-3.55, log2=1.98, pct=36%]; Oprm1[paper_only_allen_downgrade, spec=-1.67, log2=5.73, pct=82%]; Sstr2[paper_only_allen_downgrade, spec=-2.28, log2=2.47, pct=44%]; Tacr1[paper_only_allen_downgrade, spec=-6.77, log2=0.19, pct=4%]</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Cckbr(downgrade,spec=-3.22,log2=3.22); Cnr1(downgrade,spec=-10.94,log2=0.57); Crhr1(downgrade,spec=-1.36,log2=2.19); Gabbr1(downgrade,spec=-0.61,log2=8.28); Gabbr2(downgrade,spec=-1.53,log2=8.38); Gpr101(downgrade,spec=-3.42,log2=3.57); Grm5(downgrade,spec=-1.12,log2=10.36); Htr2c(downgrade,spec=-2.20,log2=7.38); Npy1r(downgrade,spec=-3.62,log2=3.71); Oprd1(downgrade,spec=-3.55,log2=1.98); Oprm1(downgrade,spec=-1.67,log2=5.73); Sstr2(downgrade,spec=-2.28,log2=2.47); Tacr1(downgrade,spec=-6.77,log2=0.19)</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H7" s="8" t="inlineStr"/>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_broadly_detectable, spec=-0.61, log2=8.28, pct=99%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.53, log2=8.38, pct=99%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm5[paper+allen_broadly_detectable, spec=-1.12, log2=10.36, pct=100%; drugs: research_only_or_none]; Oprm1[paper+allen_broadly_detectable, spec=-1.67, log2=5.73, pct=82%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Cckbr[paper_only_allen_downgrade, spec=-3.22, log2=3.22, pct=56%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-10.94, log2=0.57, pct=10%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Crhr1[paper_only_allen_downgrade, spec=-1.36, log2=2.19, pct=39%; drugs: research_only_or_none]; Gpr101[paper_only_allen_downgrade, spec=-3.42, log2=3.57, pct=57%; drugs: research_only_or_none]; Htr2c[paper_only_allen_downgrade, spec=-2.20, log2=7.38, pct=87%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Npy1r[paper_only_allen_downgrade, spec=-3.62, log2=3.71, pct=62%; drugs: research_only_or_none]; Oprd1[paper_only_allen_downgrade, spec=-3.55, log2=1.98, pct=36%; drugs: research_only_or_none]; Sstr2[paper_only_allen_downgrade, spec=-2.28, log2=2.47, pct=44%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]; Tacr1[paper_only_allen_downgrade, spec=-6.77, log2=0.19, pct=4%; drugs: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet)]</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Gabbr1, Gabbr2, Grm5, Oprm1 | paper_only: Cckbr(downgrade,spec=-3.22,log2=3.22); Cnr1(downgrade,spec=-10.94,log2=0.57); Crhr1(downgrade,spec=-1.36,log2=2.19); Gpr101(downgrade,spec=-3.42,log2=3.57); Htr2c(downgrade,spec=-2.20,log2=7.38); Npy1r(downgrade,spec=-3.62,log2=3.71); Oprd1(downgrade,spec=-3.55,log2=1.98); Sstr2(downgrade,spec=-2.28,log2=2.47); Tacr1(downgrade,spec=-6.77,log2=0.19)</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Crhr1 | clinical/research: Verucerfont; Pexacerfont; Antalarmin; Emicerfont (depression/PTSD trials mostly failed) | indication: PTSD; major depression; alcohol use disorder (mostly failed) || Gpr101 | clinical/research: research only (orphan) | indication: X-LAG / X-linked acrogigantism research || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Npy1r | clinical/research: BIBP-3226 (research antagonist) | indication: obesity; pain (preclinical) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease || Tacr1 | FDA: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet) | indication: chemotherapy-induced nausea/vomiting (CINV); postoperative nausea</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 4 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>
     <row r="8" ht="110" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>RE</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Midline thalamic glutamatergic / reuniens</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>152 RE-Xi Nox4 Glut</t>
         </is>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="8" t="n">
         <v>5450</v>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Calb2, Pcp4, Slc17a6, Spon1, Tcf7l2</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
         <is>
           <t>Gad1, Gad2</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Chrm2, Gabbr1, Gabbr2, Grm1, Grm5, Htr2a, Ntsr1, Ntsr2, Sstr2</t>
         </is>
       </c>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>Adcyap1r1[paper_only_allen_downgrade, spec=-5.37, log2=2.78, pct=46%]; Chrm2[paper_only_allen_downgrade, spec=-2.93, log2=6.27, pct=81%]; Gabbr1[paper_only_allen_downgrade, spec=-1.71, log2=9.35, pct=100%]; Gabbr2[paper_only_allen_downgrade, spec=-1.58, log2=9.23, pct=99%]; Grm1[paper_only_allen_downgrade, spec=-1.19, log2=8.82, pct=98%]; Grm5[paper_only_allen_downgrade, spec=-1.51, log2=10.02, pct=100%]; Htr2a[paper_only_allen_downgrade, spec=-3.09, log2=0.04, pct=1%]; Ntsr1[paper_only_allen_downgrade, spec=-1.23, log2=0.33, pct=6%]; Ntsr2[paper_only_allen_downgrade, spec=-9.00, log2=0.04, pct=1%]; Sstr2[paper_only_allen_downgrade, spec=-4.46, log2=0.20, pct=4%]</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-5.37,log2=2.78); Chrm2(downgrade,spec=-2.93,log2=6.27); Gabbr1(downgrade,spec=-1.71,log2=9.35); Gabbr2(downgrade,spec=-1.58,log2=9.23); Grm1(downgrade,spec=-1.19,log2=8.82); Grm5(downgrade,spec=-1.51,log2=10.02); Htr2a(downgrade,spec=-3.09,log2=0.04); Ntsr1(downgrade,spec=-1.23,log2=0.33); Ntsr2(downgrade,spec=-9.00,log2=0.04); Sstr2(downgrade,spec=-4.46,log2=0.20)</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H8" s="8" t="inlineStr"/>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_broadly_detectable, spec=-1.71, log2=9.35, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.58, log2=9.23, pct=99%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-1.19, log2=8.82, pct=98%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-1.51, log2=10.02, pct=100%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-5.37, log2=2.78, pct=46%; drugs: research_only_or_none]; Chrm2[paper_only_allen_downgrade, spec=-2.93, log2=6.27, pct=81%; drugs: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic)]; Htr2a[paper_only_allen_downgrade, spec=-3.09, log2=0.04, pct=1%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Ntsr1[paper_only_allen_downgrade, spec=-1.23, log2=0.33, pct=6%; drugs: research_only_or_none]; Ntsr2[paper_only_allen_downgrade, spec=-9.00, log2=0.04, pct=1%; drugs: research_only_or_none]; Sstr2[paper_only_allen_downgrade, spec=-4.46, log2=0.20, pct=4%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Gabbr1, Gabbr2, Grm1, Grm5 | paper_only: Adcyap1r1(downgrade,spec=-5.37,log2=2.78); Chrm2(downgrade,spec=-2.93,log2=6.27); Htr2a(downgrade,spec=-3.09,log2=0.04); Ntsr1(downgrade,spec=-1.23,log2=0.33); Ntsr2(downgrade,spec=-9.00,log2=0.04); Sstr2(downgrade,spec=-4.46,log2=0.20)</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Chrm2 | FDA: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic) | clinical/research: Methoctramine (research) | indication: Alzheimer disease; overactive bladder || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Ntsr1 | clinical/research: SR-48692 (research antagonist); SR-142948 | indication: thermal pain; addiction (preclinical) || Ntsr2 | clinical/research: research | indication: pain (preclinical) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 4 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>RE</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Midline thalamic glutamatergic / reuniens</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>149 PVT-PT Ntrk1 Glut</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="8" t="n">
         <v>9854</v>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Calb2, Pcp4, Slc17a6, Spon1, Tcf7l2</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Gad1, Gad2</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Chrm2, Gabbr1, Gabbr2, Grm1, Grm5, Htr2a, Ntsr1, Ntsr2, Sstr2</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Oprk1(spec=1.42, log2=4.18, pct=66%, status=keep); Galr1(spec=0.23, log2=2.12, pct=35%, status=keep); Oxtr(spec=0.50, log2=1.89, pct=34%, status=keep)</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>Oprk1[allen_only_keep, spec=+1.42, log2=4.18, pct=66%]; Galr1[allen_only_keep, spec=+0.23, log2=2.12, pct=35%]; Oxtr[allen_only_keep, spec=+0.50, log2=1.89, pct=34%]; Adcyap1r1[paper_only_allen_downgrade, spec=-2.91, log2=5.24, pct=81%]; Chrm2[paper_only_allen_downgrade, spec=-5.90, log2=3.30, pct=48%]; Gabbr1[paper_only_allen_downgrade, spec=-2.30, log2=8.76, pct=100%]; Gabbr2[paper_only_allen_downgrade, spec=-2.01, log2=8.80, pct=99%]; Grm1[paper_only_allen_downgrade, spec=-2.93, log2=7.07, pct=87%]; Grm5[paper_only_allen_downgrade, spec=-2.67, log2=8.86, pct=99%]; Htr2a[paper_only_allen_downgrade, spec=-3.10, log2=0.03, pct=1%]; Ntsr1[paper_only_allen_downgrade, spec=-1.24, log2=0.32, pct=6%]; Ntsr2[paper_only_allen_downgrade, spec=-8.68, log2=0.36, pct=7%]; Sstr2[paper_only_allen_downgrade, spec=-4.18, log2=0.48, pct=9%]</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-2.91,log2=5.24); Chrm2(downgrade,spec=-5.90,log2=3.30); Gabbr1(downgrade,spec=-2.30,log2=8.76); Gabbr2(downgrade,spec=-2.01,log2=8.80); Grm1(downgrade,spec=-2.93,log2=7.07); Grm5(downgrade,spec=-2.67,log2=8.86); Htr2a(downgrade,spec=-3.10,log2=0.03); Ntsr1(downgrade,spec=-1.24,log2=0.32); Ntsr2(downgrade,spec=-8.68,log2=0.36); Sstr2(downgrade,spec=-4.18,log2=0.48) | allen_only_keep: Oprk1, Galr1, Oxtr</t>
-        </is>
-      </c>
-      <c r="K9" s="7" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Oprk1[allen_only_keep, spec=+1.42, log2=4.18, pct=66%; drugs: Difelikefalin (Korsuva; FDA 2021)]; Galr1[allen_only_keep, spec=+0.23, log2=2.12, pct=35%; drugs: research_only_or_none]; Oxtr[allen_only_keep, spec=+0.50, log2=1.89, pct=34%; drugs: research_only_or_none]; Cnr1[allen_only_broadly_detectable, spec=-0.69, log2=5.48, pct=78%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Oprm1[allen_only_broadly_detectable, spec=-0.58, log2=6.85, pct=84%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Adcyap1r1[paper_only_allen_downgrade, spec=-2.91, log2=5.24, pct=81%; drugs: research_only_or_none]; Chrm2[paper_only_allen_downgrade, spec=-5.90, log2=3.30, pct=48%; drugs: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic)]; Gabbr1[paper_only_allen_downgrade, spec=-2.30, log2=8.76, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper_only_allen_downgrade, spec=-2.01, log2=8.80, pct=99%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper_only_allen_downgrade, spec=-2.93, log2=7.07, pct=87%; drugs: research_only_or_none]; Grm5[paper_only_allen_downgrade, spec=-2.67, log2=8.86, pct=99%; drugs: research_only_or_none]; Htr2a[paper_only_allen_downgrade, spec=-3.10, log2=0.03, pct=1%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Ntsr1[paper_only_allen_downgrade, spec=-1.24, log2=0.32, pct=6%; drugs: research_only_or_none]; Ntsr2[paper_only_allen_downgrade, spec=-8.68, log2=0.36, pct=7%; drugs: research_only_or_none]; Sstr2[paper_only_allen_downgrade, spec=-4.18, log2=0.48, pct=9%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>allen_only_keep: Oprk1, Galr1, Oxtr | allen_only_broadly_detectable: Cnr1, Oprm1 | paper_only: Adcyap1r1(downgrade,spec=-2.91,log2=5.24); Chrm2(downgrade,spec=-5.90,log2=3.30); Gabbr1(downgrade,spec=-2.30,log2=8.76); Gabbr2(downgrade,spec=-2.01,log2=8.80); Grm1(downgrade,spec=-2.93,log2=7.07); Grm5(downgrade,spec=-2.67,log2=8.86); Htr2a(downgrade,spec=-3.10,log2=0.03); Ntsr1(downgrade,spec=-1.24,log2=0.32); Ntsr2(downgrade,spec=-8.68,log2=0.36); Sstr2(downgrade,spec=-4.18,log2=0.48)</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>Oprk1 | FDA: Difelikefalin (Korsuva; FDA 2021) | clinical/research: Nalfurafine (Japan); Buprenorphine (mixed); CR845 | indication: uremic pruritus (Difelikefalin); depression research || Galr1 | clinical/research: research only | indication: epilepsy; depression (preclinical) || Oxtr | clinical/research: Intranasal oxytocin (autism/social trials; mostly failed); Carbetocin (Pabal - postpartum hemorrhage outside USA) | indication: autism research; social cognition; postpartum hemorrhage (Carbetocin EU) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Chrm2 | FDA: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic) | clinical/research: Methoctramine (research) | indication: Alzheimer disease; overactive bladder || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Ntsr1 | clinical/research: SR-48692 (research antagonist); SR-142948 | indication: thermal pain; addiction (preclinical) || Ntsr2 | clinical/research: research | indication: pain (preclinical) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr"/>
     </row>
     <row r="10" ht="110" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>RE</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Midline thalamic glutamatergic / reuniens</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>145 MH Tac2 Glut</t>
         </is>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="8" t="n">
         <v>7972</v>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Calb2, Pcp4, Slc17a6, Spon1, Tcf7l2</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
         <is>
           <t>Gad1, Gad2</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Chrm2, Gabbr1, Gabbr2, Grm1, Grm5, Htr2a, Ntsr1, Ntsr2, Sstr2</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Gabbr1(spec=1.44, log2=11.06, pct=100%, status=keep); Gabbr2(spec=0.83, log2=10.81, pct=99%, status=keep); Tacr1(spec=1.61, log2=6.00, pct=78%, status=keep); Sstr2(spec=2.64, log2=4.66, pct=68%, status=keep)</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>Gabbr1[paper+allen_keep, spec=+1.44, log2=11.06, pct=100%]; Gabbr2[paper+allen_keep, spec=+0.83, log2=10.81, pct=99%]; Sstr2[paper+allen_keep, spec=+2.64, log2=4.66, pct=68%]; Tacr1[allen_only_keep, spec=+1.61, log2=6.00, pct=78%]; Adcyap1r1[paper_only_allen_downgrade, spec=-7.94, log2=0.22, pct=4%]; Chrm2[paper_only_allen_downgrade, spec=-8.87, log2=0.33, pct=5%]; Grm1[paper_only_allen_downgrade, spec=-7.57, log2=2.43, pct=35%]; Grm5[paper_only_allen_downgrade, spec=-7.53, log2=3.99, pct=53%]; Htr2a[paper_only_allen_downgrade, spec=-2.68, log2=0.45, pct=7%]; Ntsr1[paper_only_allen_downgrade, spec=-1.54, log2=0.02, pct=0%]; Ntsr2[paper_only_allen_downgrade, spec=-8.96, log2=0.08, pct=2%]</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>both: Gabbr1, Gabbr2, Sstr2 | paper_only: Adcyap1r1(downgrade,spec=-7.94,log2=0.22); Chrm2(downgrade,spec=-8.87,log2=0.33); Grm1(downgrade,spec=-7.57,log2=2.43); Grm5(downgrade,spec=-7.53,log2=3.99); Htr2a(downgrade,spec=-2.68,log2=0.45); Ntsr1(downgrade,spec=-1.54,log2=0.02); Ntsr2(downgrade,spec=-8.96,log2=0.08) | allen_only_keep: Tacr1</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_keep, spec=+1.44, log2=11.06, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_keep, spec=+0.83, log2=10.81, pct=99%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Sstr2[paper+allen_keep, spec=+2.64, log2=4.66, pct=68%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]; Tacr1[allen_only_keep, spec=+1.61, log2=6.00, pct=78%; drugs: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet)]; Adcyap1r1[paper_only_allen_downgrade, spec=-7.94, log2=0.22, pct=4%; drugs: research_only_or_none]; Chrm2[paper_only_allen_downgrade, spec=-8.87, log2=0.33, pct=5%; drugs: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic)]; Grm1[paper_only_allen_downgrade, spec=-7.57, log2=2.43, pct=35%; drugs: research_only_or_none]; Grm5[paper_only_allen_downgrade, spec=-7.53, log2=3.99, pct=53%; drugs: research_only_or_none]; Htr2a[paper_only_allen_downgrade, spec=-2.68, log2=0.45, pct=7%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Ntsr1[paper_only_allen_downgrade, spec=-1.54, log2=0.02, pct=0%; drugs: research_only_or_none]; Ntsr2[paper_only_allen_downgrade, spec=-8.96, log2=0.08, pct=2%; drugs: research_only_or_none]</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Gabbr1, Gabbr2, Sstr2 | allen_only_keep: Tacr1 | paper_only: Adcyap1r1(downgrade,spec=-7.94,log2=0.22); Chrm2(downgrade,spec=-8.87,log2=0.33); Grm1(downgrade,spec=-7.57,log2=2.43); Grm5(downgrade,spec=-7.53,log2=3.99); Htr2a(downgrade,spec=-2.68,log2=0.45); Ntsr1(downgrade,spec=-1.54,log2=0.02); Ntsr2(downgrade,spec=-8.96,log2=0.08)</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease || Tacr1 | FDA: Aprepitant (Emend); Fosaprepitant; Rolapitant; Netupitant; Maropitant (vet) | indication: chemotherapy-induced nausea/vomiting (CINV); postoperative nausea || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Chrm2 | FDA: Donepezil; Rivastigmine (broad cholinesterase; indirect); Solifenacin (broad antimuscarinic) | clinical/research: Methoctramine (research) | indication: Alzheimer disease; overactive bladder || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Ntsr1 | clinical/research: SR-48692 (research antagonist); SR-142948 | indication: thermal pain; addiction (preclinical) || Ntsr2 | clinical/research: research | indication: pain (preclinical)</t>
+        </is>
+      </c>
+      <c r="N10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="110" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>LM</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Lateral mammillary excitatory</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>144 MM Foxb1 Glut</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="8" t="n">
         <v>8270</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Foxb1, Lhx5, Pou4f1</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>Slc32a1</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Avpr1a, Cckbr, Gabbr1, Gabbr2, Grm1, Hcrtr1, Hcrtr2, Mc4r, Oxtr, Sstr2</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>Adcyap1r1[paper_only_allen_downgrade, spec=-4.76, log2=2.64, pct=47%]; Avpr1a[paper_only_allen_downgrade, spec=-2.15, log2=0.01, pct=0%]; Cckbr[paper_only_allen_downgrade, spec=-4.07, log2=0.28, pct=6%]; Gabbr1[paper_only_allen_downgrade, spec=-1.00, log2=8.28, pct=98%]; Gabbr2[paper_only_allen_downgrade, spec=-1.75, log2=8.35, pct=97%]; Grm1[paper_only_allen_downgrade, spec=-0.13, log2=9.71, pct=100%]; Hcrtr1[paper_only_allen_downgrade, spec=-1.61, log2=0.02, pct=0%]; Hcrtr2[paper_only_allen_downgrade, spec=-4.36, log2=1.25, pct=21%]; Mc4r[paper_only_allen_downgrade, spec=-1.20, log2=0.00, pct=0%]; Oxtr[paper_only_allen_downgrade, spec=-3.63, log2=0.01, pct=0%]; Sstr2[paper_only_allen_downgrade, spec=-2.19, log2=0.37, pct=7%]</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-4.76,log2=2.64); Avpr1a(downgrade,spec=-2.15,log2=0.01); Cckbr(downgrade,spec=-4.07,log2=0.28); Gabbr1(downgrade,spec=-1.00,log2=8.28); Gabbr2(downgrade,spec=-1.75,log2=8.35); Grm1(downgrade,spec=-0.13,log2=9.71); Hcrtr1(downgrade,spec=-1.61,log2=0.02); Hcrtr2(downgrade,spec=-4.36,log2=1.25); Mc4r(downgrade,spec=-1.20,log2=0.00); Oxtr(downgrade,spec=-3.63,log2=0.01); Sstr2(downgrade,spec=-2.19,log2=0.37)</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H11" s="8" t="inlineStr"/>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1[paper+allen_broadly_detectable, spec=-1.00, log2=8.28, pct=98%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.75, log2=8.35, pct=97%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-0.13, log2=9.71, pct=100%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-4.76, log2=2.64, pct=47%; drugs: research_only_or_none]; Avpr1a[paper_only_allen_downgrade, spec=-2.15, log2=0.01, pct=0%; drugs: research_only_or_none]; Cckbr[paper_only_allen_downgrade, spec=-4.07, log2=0.28, pct=6%; drugs: research_only_or_none]; Hcrtr1[paper_only_allen_downgrade, spec=-1.61, log2=0.02, pct=0%; drugs: research_only_or_none]; Hcrtr2[paper_only_allen_downgrade, spec=-4.36, log2=1.25, pct=21%; drugs: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2]; Mc4r[paper_only_allen_downgrade, spec=-1.20, log2=0.00, pct=0%; drugs: Setmelanotide (Imcivree; FDA 2020)]; Oxtr[paper_only_allen_downgrade, spec=-3.63, log2=0.01, pct=0%; drugs: research_only_or_none]; Sstr2[paper_only_allen_downgrade, spec=-2.19, log2=0.37, pct=7%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Gabbr1, Gabbr2, Grm1 | paper_only: Adcyap1r1(downgrade,spec=-4.76,log2=2.64); Avpr1a(downgrade,spec=-2.15,log2=0.01); Cckbr(downgrade,spec=-4.07,log2=0.28); Hcrtr1(downgrade,spec=-1.61,log2=0.02); Hcrtr2(downgrade,spec=-4.36,log2=1.25); Mc4r(downgrade,spec=-1.20,log2=0.00); Oxtr(downgrade,spec=-3.63,log2=0.01); Sstr2(downgrade,spec=-2.19,log2=0.37)</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Avpr1a | clinical/research: Balovaptan / RG7314 (autism trials FAILED 2020) | indication: autism social-cognition trials || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Hcrtr1 | clinical/research: SB-334867 (research selective antagonist) | indication: addiction; anxiety (preclinical) || Hcrtr2 | FDA: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2 | clinical/research: JNJ-42847922 (selective OX2R) | indication: insomnia || Mc4r | FDA: Setmelanotide (Imcivree; FDA 2020) | clinical/research: Bremelanotide (Vyleesi PT-141 - MC4 partial agonist for HSDD) | indication: rare genetic obesity (POMC/LEPR/PCSK1 deficiency; Bardet-Biedl syndrome); female sexual dysfunction (Bremelanotide) || Oxtr | clinical/research: Intranasal oxytocin (autism/social trials; mostly failed); Carbetocin (Pabal - postpartum hemorrhage outside USA) | indication: autism research; social cognition; postpartum hemorrhage (Carbetocin EU) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 3 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>LM</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Lateral mammillary excitatory</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>143 MM-ant Foxb1 Glut</t>
         </is>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="8" t="n">
         <v>5437</v>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Foxb1, Lhx5, Pou4f1</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Slc32a1</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Avpr1a, Cckbr, Gabbr1, Gabbr2, Grm1, Hcrtr1, Hcrtr2, Mc4r, Oxtr, Sstr2</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>Htr2a(spec=1.70, log2=5.18, pct=73%, status=keep)</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
-        <is>
-          <t>Htr2a[allen_only_keep, spec=+1.70, log2=5.18, pct=73%]; Adcyap1r1[paper_only_allen_downgrade, spec=-4.46, log2=2.93, pct=49%]; Avpr1a[paper_only_allen_downgrade, spec=-2.15, log2=0.00, pct=0%]; Cckbr[paper_only_allen_downgrade, spec=-2.99, log2=1.36, pct=24%]; Gabbr1[paper_only_allen_downgrade, spec=-1.09, log2=8.19, pct=97%]; Gabbr2[paper_only_allen_downgrade, spec=-1.74, log2=8.36, pct=97%]; Grm1[paper_only_allen_downgrade, spec=-0.99, log2=8.85, pct=97%]; Hcrtr1[paper_only_allen_downgrade, spec=-1.58, log2=0.05, pct=1%]; Hcrtr2[paper_only_allen_downgrade, spec=-4.97, log2=0.64, pct=11%]; Mc4r[paper_only_allen_downgrade, spec=-1.20, log2=0.01, pct=0%]; Oxtr[paper_only_allen_downgrade, spec=-3.63, log2=0.00, pct=0%]; Sstr2[paper_only_allen_downgrade, spec=-1.93, log2=0.63, pct=12%]</t>
-        </is>
-      </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-4.46,log2=2.93); Avpr1a(downgrade,spec=-2.15,log2=0.00); Cckbr(downgrade,spec=-2.99,log2=1.36); Gabbr1(downgrade,spec=-1.09,log2=8.19); Gabbr2(downgrade,spec=-1.74,log2=8.36); Grm1(downgrade,spec=-0.99,log2=8.85); Hcrtr1(downgrade,spec=-1.58,log2=0.05); Hcrtr2(downgrade,spec=-4.97,log2=0.64); Mc4r(downgrade,spec=-1.20,log2=0.01); Oxtr(downgrade,spec=-3.63,log2=0.00); Sstr2(downgrade,spec=-1.93,log2=0.63) | allen_only_keep: Htr2a</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Htr2a[allen_only_keep, spec=+1.70, log2=5.18, pct=73%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Gabbr1[paper+allen_broadly_detectable, spec=-1.09, log2=8.19, pct=97%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.74, log2=8.36, pct=97%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-0.99, log2=8.85, pct=97%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-4.46, log2=2.93, pct=49%; drugs: research_only_or_none]; Avpr1a[paper_only_allen_downgrade, spec=-2.15, log2=0.00, pct=0%; drugs: research_only_or_none]; Cckbr[paper_only_allen_downgrade, spec=-2.99, log2=1.36, pct=24%; drugs: research_only_or_none]; Hcrtr1[paper_only_allen_downgrade, spec=-1.58, log2=0.05, pct=1%; drugs: research_only_or_none]; Hcrtr2[paper_only_allen_downgrade, spec=-4.97, log2=0.64, pct=11%; drugs: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2]; Mc4r[paper_only_allen_downgrade, spec=-1.20, log2=0.01, pct=0%; drugs: Setmelanotide (Imcivree; FDA 2020)]; Oxtr[paper_only_allen_downgrade, spec=-3.63, log2=0.00, pct=0%; drugs: research_only_or_none]; Sstr2[paper_only_allen_downgrade, spec=-1.93, log2=0.63, pct=12%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>allen_only_keep: Htr2a | paper+broadly_detectable: Gabbr1, Gabbr2, Grm1 | paper_only: Adcyap1r1(downgrade,spec=-4.46,log2=2.93); Avpr1a(downgrade,spec=-2.15,log2=0.00); Cckbr(downgrade,spec=-2.99,log2=1.36); Hcrtr1(downgrade,spec=-1.58,log2=0.05); Hcrtr2(downgrade,spec=-4.97,log2=0.64); Mc4r(downgrade,spec=-1.20,log2=0.01); Oxtr(downgrade,spec=-3.63,log2=0.00); Sstr2(downgrade,spec=-1.93,log2=0.63)</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Avpr1a | clinical/research: Balovaptan / RG7314 (autism trials FAILED 2020) | indication: autism social-cognition trials || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Hcrtr1 | clinical/research: SB-334867 (research selective antagonist) | indication: addiction; anxiety (preclinical) || Hcrtr2 | FDA: Suvorexant (Belsomra); Lemborexant (Dayvigo); Daridorexant (Quviviq) - all Dual Orexin Receptor Antagonists hitting both 1+2 | clinical/research: JNJ-42847922 (selective OX2R) | indication: insomnia || Mc4r | FDA: Setmelanotide (Imcivree; FDA 2020) | clinical/research: Bremelanotide (Vyleesi PT-141 - MC4 partial agonist for HSDD) | indication: rare genetic obesity (POMC/LEPR/PCSK1 deficiency; Bardet-Biedl syndrome); female sexual dysfunction (Bremelanotide) || Oxtr | clinical/research: Intranasal oxytocin (autism/social trials; mostly failed); Carbetocin (Pabal - postpartum hemorrhage outside USA) | indication: autism research; social cognition; postpartum hemorrhage (Carbetocin EU) || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="110" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>ORBm</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>L2/3 IT excitatory</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>007 L2/3 IT CTX Glut</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="8" t="n">
         <v>8869</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Cdh13, Cux1, Cux2, Rorb, Satb2, Slc17a7</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>Gad1, Slc32a1</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Cckbr, Cnr1, Gabbr1, Gabbr2, Grm1, Grm5, Htr2a, Npy1r, Oprd1, Oprm1, Sstr2</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>Cckbr(spec=0.08, log2=4.87, pct=73%, status=keep)</t>
         </is>
       </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Cckbr[paper+allen_keep, spec=+0.08, log2=4.87, pct=73%]; Cnr1[paper_only_allen_downgrade, spec=-6.50, log2=5.66, pct=83%]; Gabbr1[paper_only_allen_downgrade, spec=-0.34, log2=8.47, pct=99%]; Gabbr2[paper_only_allen_downgrade, spec=-0.59, log2=9.02, pct=100%]; Grm1[paper_only_allen_downgrade, spec=-0.90, log2=7.68, pct=94%]; Grm5[paper_only_allen_downgrade, spec=-0.82, log2=10.48, pct=100%]; Htr2a[paper_only_allen_downgrade, spec=-4.91, log2=2.84, pct=45%]; Npy1r[paper_only_allen_downgrade, spec=-2.34, log2=4.06, pct=64%]; Oprd1[paper_only_allen_downgrade, spec=-3.19, log2=1.39, pct=25%]; Oprm1[paper_only_allen_downgrade, spec=-3.60, log2=2.01, pct=35%]; Sstr2[paper_only_allen_downgrade, spec=-7.42, log2=0.37, pct=7%]</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr">
-        <is>
-          <t>both: Cckbr | paper_only: Cnr1(downgrade,spec=-6.50,log2=5.66); Gabbr1(downgrade,spec=-0.34,log2=8.47); Gabbr2(downgrade,spec=-0.59,log2=9.02); Grm1(downgrade,spec=-0.90,log2=7.68); Grm5(downgrade,spec=-0.82,log2=10.48); Htr2a(downgrade,spec=-4.91,log2=2.84); Npy1r(downgrade,spec=-2.34,log2=4.06); Oprd1(downgrade,spec=-3.19,log2=1.39); Oprm1(downgrade,spec=-3.60,log2=2.01); Sstr2(downgrade,spec=-7.42,log2=0.37)</t>
-        </is>
-      </c>
-      <c r="K13" s="7" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Cckbr[paper+allen_keep, spec=+0.08, log2=4.87, pct=73%; drugs: research_only_or_none]; Gabbr1[paper+allen_broadly_detectable, spec=-0.34, log2=8.47, pct=99%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-0.59, log2=9.02, pct=100%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-0.90, log2=7.68, pct=94%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-0.82, log2=10.48, pct=100%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-6.50, log2=5.66, pct=83%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Htr2a[paper_only_allen_downgrade, spec=-4.91, log2=2.84, pct=45%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Npy1r[paper_only_allen_downgrade, spec=-2.34, log2=4.06, pct=64%; drugs: research_only_or_none]; Oprd1[paper_only_allen_downgrade, spec=-3.19, log2=1.39, pct=25%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-3.60, log2=2.01, pct=35%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Sstr2[paper_only_allen_downgrade, spec=-7.42, log2=0.37, pct=7%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Cckbr | paper+broadly_detectable: Gabbr1, Gabbr2, Grm1, Grm5 | paper_only: Cnr1(downgrade,spec=-6.50,log2=5.66); Htr2a(downgrade,spec=-4.91,log2=2.84); Npy1r(downgrade,spec=-2.34,log2=4.06); Oprd1(downgrade,spec=-3.19,log2=1.39); Oprm1(downgrade,spec=-3.60,log2=2.01); Sstr2(downgrade,spec=-7.42,log2=0.37)</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Npy1r | clinical/research: BIBP-3226 (research antagonist) | indication: obesity; pain (preclinical) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr"/>
     </row>
     <row r="14" ht="110" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>AId</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Upper-layer IT excitatory</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>007 L2/3 IT CTX Glut</t>
         </is>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="8" t="n">
         <v>7697</v>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Cux1, Cux2, Rorb, Slc17a7</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>Gad1, Slc32a1</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Cckbr, Cnr1, Gabbr1, Gabbr2, Grm5, Htr2a, Npy1r, Oprd1, Oprm1, Sstr2</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Gpr88(spec=0.33, log2=4.77, pct=74%, status=keep)</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
-        <is>
-          <t>Gpr88[allen_only_keep, spec=+0.33, log2=4.77, pct=74%]; Cckbr[paper_only_allen_downgrade, spec=-1.05, log2=4.52, pct=71%]; Cnr1[paper_only_allen_downgrade, spec=-6.83, log2=5.24, pct=81%]; Gabbr1[paper_only_allen_downgrade, spec=-0.76, log2=8.52, pct=100%]; Gabbr2[paper_only_allen_downgrade, spec=-0.45, log2=9.12, pct=100%]; Grm5[paper_only_allen_downgrade, spec=-0.28, log2=10.52, pct=100%]; Htr2a[paper_only_allen_downgrade, spec=-2.79, log2=4.48, pct=69%]; Npy1r[paper_only_allen_downgrade, spec=-2.04, log2=3.75, pct=62%]; Oprd1[paper_only_allen_downgrade, spec=-2.71, log2=1.63, pct=30%]; Oprm1[paper_only_allen_downgrade, spec=-4.68, log2=2.21, pct=39%]; Sstr2[paper_only_allen_downgrade, spec=-6.30, log2=0.56, pct=11%]</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Cckbr(downgrade,spec=-1.05,log2=4.52); Cnr1(downgrade,spec=-6.83,log2=5.24); Gabbr1(downgrade,spec=-0.76,log2=8.52); Gabbr2(downgrade,spec=-0.45,log2=9.12); Grm5(downgrade,spec=-0.28,log2=10.52); Htr2a(downgrade,spec=-2.79,log2=4.48); Npy1r(downgrade,spec=-2.04,log2=3.75); Oprd1(downgrade,spec=-2.71,log2=1.63); Oprm1(downgrade,spec=-4.68,log2=2.21); Sstr2(downgrade,spec=-6.30,log2=0.56) | allen_only_keep: Gpr88</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="inlineStr"/>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Gpr88[allen_only_keep, spec=+0.33, log2=4.77, pct=74%; drugs: research_only_or_none]; Cckbr[paper+allen_broadly_detectable, spec=-1.05, log2=4.52, pct=71%; drugs: research_only_or_none]; Gabbr1[paper+allen_broadly_detectable, spec=-0.76, log2=8.52, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-0.45, log2=9.12, pct=100%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm5[paper+allen_broadly_detectable, spec=-0.28, log2=10.52, pct=100%; drugs: research_only_or_none]; Grm1[allen_only_broadly_detectable, spec=-0.92, log2=7.76, pct=96%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-6.83, log2=5.24, pct=81%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Htr2a[paper_only_allen_downgrade, spec=-2.79, log2=4.48, pct=69%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Npy1r[paper_only_allen_downgrade, spec=-2.04, log2=3.75, pct=62%; drugs: research_only_or_none]; Oprd1[paper_only_allen_downgrade, spec=-2.71, log2=1.63, pct=30%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-4.68, log2=2.21, pct=39%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Sstr2[paper_only_allen_downgrade, spec=-6.30, log2=0.56, pct=11%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>allen_only_keep: Gpr88 | paper+broadly_detectable: Cckbr, Gabbr1, Gabbr2, Grm5 | allen_only_broadly_detectable: Grm1 | paper_only: Cnr1(downgrade,spec=-6.83,log2=5.24); Htr2a(downgrade,spec=-2.79,log2=4.48); Npy1r(downgrade,spec=-2.04,log2=3.75); Oprd1(downgrade,spec=-2.71,log2=1.63); Oprm1(downgrade,spec=-4.68,log2=2.21); Sstr2(downgrade,spec=-6.30,log2=0.56)</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>Gpr88 | clinical/research: RTI-13951-33 (research agonist) | indication: obsessive-compulsive disorder; addiction (preclinical) || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Npy1r | clinical/research: BIBP-3226 (research antagonist) | indication: obesity; pain (preclinical) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="110" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>AId</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Upper-layer IT excitatory</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>006 L4/5 IT CTX Glut</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="8" t="n">
         <v>12177</v>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Cux1, Cux2, Rorb, Slc17a7</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>Gad1, Slc32a1</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Cckbr, Cnr1, Gabbr1, Gabbr2, Grm5, Htr2a, Npy1r, Oprd1, Oprm1, Sstr2</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>Crhr1(spec=0.13, log2=3.94, pct=64%, status=keep)</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>Crhr1[allen_only_keep, spec=+0.13, log2=3.94, pct=64%]; Cckbr[paper_only_allen_downgrade, spec=-1.60, log2=3.96, pct=64%]; Cnr1[paper_only_allen_downgrade, spec=-5.56, log2=6.51, pct=89%]; Gabbr1[paper_only_allen_downgrade, spec=-0.58, log2=8.70, pct=100%]; Gabbr2[paper_only_allen_downgrade, spec=-0.61, log2=8.96, pct=99%]; Grm5[paper_only_allen_downgrade, spec=-1.07, log2=9.73, pct=100%]; Htr2a[paper_only_allen_downgrade, spec=-0.69, log2=6.59, pct=91%]; Npy1r[paper_only_allen_downgrade, spec=-2.45, log2=3.34, pct=56%]; Oprd1[paper_only_allen_downgrade, spec=-3.12, log2=1.22, pct=22%]; Oprm1[paper_only_allen_downgrade, spec=-4.84, log2=2.05, pct=36%]; Sstr2[paper_only_allen_downgrade, spec=-5.69, log2=1.16, pct=20%]</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Cckbr(downgrade,spec=-1.60,log2=3.96); Cnr1(downgrade,spec=-5.56,log2=6.51); Gabbr1(downgrade,spec=-0.58,log2=8.70); Gabbr2(downgrade,spec=-0.61,log2=8.96); Grm5(downgrade,spec=-1.07,log2=9.73); Htr2a(downgrade,spec=-0.69,log2=6.59); Npy1r(downgrade,spec=-2.45,log2=3.34); Oprd1(downgrade,spec=-3.12,log2=1.22); Oprm1(downgrade,spec=-4.84,log2=2.05); Sstr2(downgrade,spec=-5.69,log2=1.16) | allen_only_keep: Crhr1</t>
-        </is>
-      </c>
-      <c r="K15" s="7" t="inlineStr"/>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Crhr1[allen_only_keep, spec=+0.13, log2=3.94, pct=64%; drugs: research_only_or_none]; Gabbr1[paper+allen_broadly_detectable, spec=-0.58, log2=8.70, pct=100%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-0.61, log2=8.96, pct=99%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm5[paper+allen_broadly_detectable, spec=-1.07, log2=9.73, pct=100%; drugs: research_only_or_none]; Htr2a[paper+allen_broadly_detectable, spec=-0.69, log2=6.59, pct=91%; drugs: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine]; Htr1f[allen_only_broadly_detectable, spec=-1.26, log2=6.28, pct=86%; drugs: Lasmiditan (Reyvow; FDA 2019)]; Cckbr[paper_only_allen_downgrade, spec=-1.60, log2=3.96, pct=64%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-5.56, log2=6.51, pct=89%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Npy1r[paper_only_allen_downgrade, spec=-2.45, log2=3.34, pct=56%; drugs: research_only_or_none]; Oprd1[paper_only_allen_downgrade, spec=-3.12, log2=1.22, pct=22%; drugs: research_only_or_none]; Oprm1[paper_only_allen_downgrade, spec=-4.84, log2=2.05, pct=36%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Sstr2[paper_only_allen_downgrade, spec=-5.69, log2=1.16, pct=20%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>allen_only_keep: Crhr1 | paper+broadly_detectable: Gabbr1, Gabbr2, Grm5, Htr2a | allen_only_broadly_detectable: Htr1f | paper_only: Cckbr(downgrade,spec=-1.60,log2=3.96); Cnr1(downgrade,spec=-5.56,log2=6.51); Npy1r(downgrade,spec=-2.45,log2=3.34); Oprd1(downgrade,spec=-3.12,log2=1.22); Oprm1(downgrade,spec=-4.84,log2=2.05); Sstr2(downgrade,spec=-5.69,log2=1.16)</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>Crhr1 | clinical/research: Verucerfont; Pexacerfont; Antalarmin; Emicerfont (depression/PTSD trials mostly failed) | indication: PTSD; major depression; alcohol use disorder (mostly failed) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Htr2a | FDA: Pimavanserin (Nuplazid; FDA Parkinson psychosis); Risperidone; Olanzapine; Aripiprazole; Trazodone; Mirtazapine; Quetiapine; Clozapine | clinical/research: Psilocybin (FDA breakthrough for depression); MDMA-assisted therapy; Ketanserin (Europe) | indication: Parkinson psychosis; schizophrenia; treatment-resistant depression (psychedelic trials) || Htr1f | FDA: Lasmiditan (Reyvow; FDA 2019) | indication: migraine (acute attack) || Cckbr | clinical/research: Netazepide / YF476 (research antagonist) | indication: acid hypersecretion; anxiety (preclinical) || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Npy1r | clinical/research: BIBP-3226 (research antagonist) | indication: obesity; pain (preclinical) || Oprd1 | clinical/research: DPDPE; ADL-5859; SNC-80 (research) | indication: depression; chronic pain (preclinical) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="110" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>CA1 pyramidal</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>016 CA1-ProS Glut</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="8" t="n">
         <v>24868</v>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Fibcd1, Mpped1, Pou3f1, Slc17a7, Spink8, Wfs1</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Calb1, Cnih3, Prox1, Rgs14</t>
         </is>
       </c>
-      <c r="G16" s="7" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Cnr1, Drd1, Drd2, Gabbr1, Gabbr2, Grm1, Grm5, Htr1a, Htr1b, Htr2c, Oprm1, Sstr2</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>Htr1a(spec=0.96, log2=3.33, pct=55%, status=keep); Mc4r(spec=0.08, log2=1.12, pct=21%, status=keep)</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
-        <is>
-          <t>Htr1a[paper+allen_keep, spec=+0.96, log2=3.33, pct=55%]; Mc4r[allen_only_keep, spec=+0.08, log2=1.12, pct=21%]; Adcyap1r1[paper_only_allen_downgrade, spec=-4.69, log2=1.63, pct=29%]; Cnr1[paper_only_allen_downgrade, spec=-7.05, log2=5.38, pct=80%]; Drd1[paper_only_allen_downgrade, spec=-1.77, log2=0.02, pct=0%]; Drd2[paper_only_allen_downgrade, spec=-1.50, log2=0.01, pct=0%]; Gabbr1[paper_only_allen_downgrade, spec=-0.45, log2=8.70, pct=99%]; Gabbr2[paper_only_allen_downgrade, spec=-1.96, log2=7.93, pct=96%]; Grm1[paper_only_allen_downgrade, spec=-1.93, log2=6.56, pct=85%]; Grm5[paper_only_allen_downgrade, spec=-0.36, log2=10.79, pct=100%]; Htr1b[paper_only_allen_downgrade, spec=-1.27, log2=2.14, pct=38%]; Htr2c[paper_only_allen_downgrade, spec=-10.14, log2=1.80, pct=29%]; Oprm1[paper_only_allen_downgrade, spec=-6.78, log2=0.18, pct=3%]; Sstr2[paper_only_allen_downgrade, spec=-3.27, log2=0.51, pct=10%]</t>
-        </is>
-      </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>both: Htr1a | paper_only: Adcyap1r1(downgrade,spec=-4.69,log2=1.63); Cnr1(downgrade,spec=-7.05,log2=5.38); Drd1(downgrade,spec=-1.77,log2=0.02); Drd2(downgrade,spec=-1.50,log2=0.01); Gabbr1(downgrade,spec=-0.45,log2=8.70); Gabbr2(downgrade,spec=-1.96,log2=7.93); Grm1(downgrade,spec=-1.93,log2=6.56); Grm5(downgrade,spec=-0.36,log2=10.79); Htr1b(downgrade,spec=-1.27,log2=2.14); Htr2c(downgrade,spec=-10.14,log2=1.80); Oprm1(downgrade,spec=-6.78,log2=0.18); Sstr2(downgrade,spec=-3.27,log2=0.51) | allen_only_keep: Mc4r</t>
-        </is>
-      </c>
-      <c r="K16" s="7" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Htr1a[paper+allen_keep, spec=+0.96, log2=3.33, pct=55%; drugs: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone]; Mc4r[allen_only_keep, spec=+0.08, log2=1.12, pct=21%; drugs: Setmelanotide (Imcivree; FDA 2020)]; Gabbr1[paper+allen_broadly_detectable, spec=-0.45, log2=8.70, pct=99%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.96, log2=7.93, pct=96%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-1.93, log2=6.56, pct=85%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-0.36, log2=10.79, pct=100%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-4.69, log2=1.63, pct=29%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-7.05, log2=5.38, pct=80%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Drd1[paper_only_allen_downgrade, spec=-1.77, log2=0.02, pct=0%; drugs: Apomorphine (mixed); Pergolide (partial)]; Drd2[paper_only_allen_downgrade, spec=-1.50, log2=0.01, pct=0%; drugs: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect)]; Htr1b[paper_only_allen_downgrade, spec=-1.27, log2=2.14, pct=38%; drugs: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan]; Htr2c[paper_only_allen_downgrade, spec=-10.14, log2=1.80, pct=29%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]; Oprm1[paper_only_allen_downgrade, spec=-6.78, log2=0.18, pct=3%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]; Sstr2[paper_only_allen_downgrade, spec=-3.27, log2=0.51, pct=10%; drugs: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy)]</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Htr1a | allen_only_keep: Mc4r | paper+broadly_detectable: Gabbr1, Gabbr2, Grm1, Grm5 | paper_only: Adcyap1r1(downgrade,spec=-4.69,log2=1.63); Cnr1(downgrade,spec=-7.05,log2=5.38); Drd1(downgrade,spec=-1.77,log2=0.02); Drd2(downgrade,spec=-1.50,log2=0.01); Htr1b(downgrade,spec=-1.27,log2=2.14); Htr2c(downgrade,spec=-10.14,log2=1.80); Oprm1(downgrade,spec=-6.78,log2=0.18); Sstr2(downgrade,spec=-3.27,log2=0.51)</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>Htr1a | FDA: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone | clinical/research: NLX-101 (depression) | indication: generalized anxiety; major depression || Mc4r | FDA: Setmelanotide (Imcivree; FDA 2020) | clinical/research: Bremelanotide (Vyleesi PT-141 - MC4 partial agonist for HSDD) | indication: rare genetic obesity (POMC/LEPR/PCSK1 deficiency; Bardet-Biedl syndrome); female sexual dysfunction (Bremelanotide) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Drd1 | FDA: Apomorphine (mixed); Pergolide (partial) | clinical/research: SKF-81297; SKF-38393 (research agonists); SCH-23390 (antagonist) | indication: Parkinson disease; addiction research || Drd2 | FDA: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect) | clinical/research: many | indication: schizophrenia; bipolar; Parkinson disease; hyperprolactinemia || Htr1b | FDA: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan | indication: migraine (acute attack) || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia || Sstr2 | FDA: Octreotide; Lanreotide; Pasireotide (broad SSTR); Lutetium Lu-177 dotatate (radiotherapy) | indication: acromegaly; neuroendocrine tumors (NETs); Cushing disease</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="110" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>CA2 pyramidal</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>025 CA2-FC-IG Glut</t>
         </is>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="8" t="n">
         <v>327</v>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Amigo2, Avpr1b, Cacng5, Map3k15, Pcp4, Rgs14, Slc17a7</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>Cnih3, Prox1, Wfs1</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Avpr1a, Avpr1b, Cnr1, Drd1, Gabbr1, Gabbr2, Grm1, Grm5, Htr1a, Oxtr</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>Avpr1b(spec=0.77, log2=0.81, pct=17%, status=keep_validate_spatially)</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>Avpr1b[paper+allen_keep, spec=+0.77, log2=0.81, pct=17%]; Avpr1a[paper_only_allen_downgrade, spec=-0.08, log2=0.03, pct=1%]; Cnr1[paper_only_allen_downgrade, spec=-6.66, log2=5.77, pct=87%]; Drd1[paper_only_allen_downgrade, spec=-0.64, log2=1.15, pct=21%]; Gabbr1[paper_only_allen_downgrade, spec=-0.99, log2=8.16, pct=99%]; Gabbr2[paper_only_allen_downgrade, spec=-1.64, log2=8.25, pct=97%]; Grm1[paper_only_allen_downgrade, spec=-2.06, log2=6.43, pct=89%]; Grm5[paper_only_allen_downgrade, spec=-0.81, log2=10.35, pct=100%]; Htr1a[paper_only_allen_downgrade, spec=-3.00, log2=0.33, pct=7%]; Oxtr[paper_only_allen_downgrade, spec=-0.07, log2=1.27, pct=24%]</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>both: Avpr1b | paper_only: Avpr1a(downgrade,spec=-0.08,log2=0.03); Cnr1(downgrade,spec=-6.66,log2=5.77); Drd1(downgrade,spec=-0.64,log2=1.15); Gabbr1(downgrade,spec=-0.99,log2=8.16); Gabbr2(downgrade,spec=-1.64,log2=8.25); Grm1(downgrade,spec=-2.06,log2=6.43); Grm5(downgrade,spec=-0.81,log2=10.35); Htr1a(downgrade,spec=-3.00,log2=0.33); Oxtr(downgrade,spec=-0.07,log2=1.27)</t>
-        </is>
-      </c>
-      <c r="K17" s="7" t="inlineStr"/>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Avpr1b[paper+allen_keep, spec=+0.77, log2=0.81, pct=17%; drugs: research_only_or_none]; Gabbr1[paper+allen_broadly_detectable, spec=-0.99, log2=8.16, pct=99%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-1.64, log2=8.25, pct=97%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm5[paper+allen_broadly_detectable, spec=-0.81, log2=10.35, pct=100%; drugs: research_only_or_none]; Avpr1a[paper_only_allen_downgrade, spec=-0.08, log2=0.03, pct=1%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-6.66, log2=5.77, pct=87%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Drd1[paper_only_allen_downgrade, spec=-0.64, log2=1.15, pct=21%; drugs: Apomorphine (mixed); Pergolide (partial)]; Grm1[paper_only_allen_downgrade, spec=-2.06, log2=6.43, pct=89%; drugs: research_only_or_none]; Htr1a[paper_only_allen_downgrade, spec=-3.00, log2=0.33, pct=7%; drugs: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone]; Oxtr[paper_only_allen_downgrade, spec=-0.07, log2=1.27, pct=24%; drugs: research_only_or_none]</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>both_keep: Avpr1b | paper+broadly_detectable: Gabbr1, Gabbr2, Grm5 | paper_only: Avpr1a(downgrade,spec=-0.08,log2=0.03); Cnr1(downgrade,spec=-6.66,log2=5.77); Drd1(downgrade,spec=-0.64,log2=1.15); Grm1(downgrade,spec=-2.06,log2=6.43); Htr1a(downgrade,spec=-3.00,log2=0.33); Oxtr(downgrade,spec=-0.07,log2=1.27)</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>Avpr1b | clinical/research: Nelivaptan / SSR149415 (depression trials failed); ABT-558 | indication: major depression; PTSD; anxiety (failed/discontinued) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Avpr1a | clinical/research: Balovaptan / RG7314 (autism trials FAILED 2020) | indication: autism social-cognition trials || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Drd1 | FDA: Apomorphine (mixed); Pergolide (partial) | clinical/research: SKF-81297; SKF-38393 (research agonists); SCH-23390 (antagonist) | indication: Parkinson disease; addiction research || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Htr1a | FDA: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone | clinical/research: NLX-101 (depression) | indication: generalized anxiety; major depression || Oxtr | clinical/research: Intranasal oxytocin (autism/social trials; mostly failed); Carbetocin (Pabal - postpartum hemorrhage outside USA) | indication: autism research; social cognition; postpartum hemorrhage (Carbetocin EU)</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr"/>
     </row>
     <row r="18" ht="110" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>CA3 pyramidal</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>017 CA3 Glut</t>
         </is>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="8" t="n">
         <v>4799</v>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Calb2, Cnih3, Coch, Lct, Slc17a7</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Prox1, Rgs14, Wfs1</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Cnr1, Drd2, Gabbr1, Gabbr2, Grm1, Grm5, Htr1a, Htr1b, Oprm1</t>
         </is>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>Npy2r(spec=2.24, log2=5.61, pct=85%, status=keep); Hcrtr1(spec=0.01, log2=0.28, pct=6%, status=candidate_to_validate)</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
-        <is>
-          <t>Npy2r[allen_only_keep, spec=+2.24, log2=5.61, pct=85%]; Hcrtr1[allen_only_keep, spec=+0.01, log2=0.28, pct=6%]; Adcyap1r1[paper_only_allen_downgrade, spec=-5.28, log2=1.04, pct=20%]; Cnr1[paper_only_allen_downgrade, spec=-5.87, log2=6.56, pct=94%]; Drd2[paper_only_allen_downgrade, spec=-1.32, log2=0.19, pct=3%]; Gabbr1[paper_only_allen_downgrade, spec=-0.90, log2=8.25, pct=99%]; Gabbr2[paper_only_allen_downgrade, spec=-0.87, log2=9.02, pct=100%]; Grm1[paper_only_allen_downgrade, spec=-1.10, log2=7.39, pct=93%]; Grm5[paper_only_allen_downgrade, spec=-0.96, log2=10.19, pct=100%]; Htr1a[paper_only_allen_downgrade, spec=-1.93, log2=1.39, pct=28%]; Htr1b[paper_only_allen_downgrade, spec=-3.36, log2=0.05, pct=1%]; Oprm1[paper_only_allen_downgrade, spec=-6.77, log2=0.19, pct=4%]</t>
-        </is>
-      </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-5.28,log2=1.04); Cnr1(downgrade,spec=-5.87,log2=6.56); Drd2(downgrade,spec=-1.32,log2=0.19); Gabbr1(downgrade,spec=-0.90,log2=8.25); Gabbr2(downgrade,spec=-0.87,log2=9.02); Grm1(downgrade,spec=-1.10,log2=7.39); Grm5(downgrade,spec=-0.96,log2=10.19); Htr1a(downgrade,spec=-1.93,log2=1.39); Htr1b(downgrade,spec=-3.36,log2=0.05); Oprm1(downgrade,spec=-6.77,log2=0.19) | allen_only_keep: Npy2r, Hcrtr1</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Npy2r[allen_only_keep, spec=+2.24, log2=5.61, pct=85%; drugs: research_only_or_none]; Hcrtr1[allen_only_keep, spec=+0.01, log2=0.28, pct=6%; drugs: research_only_or_none]; Gabbr1[paper+allen_broadly_detectable, spec=-0.90, log2=8.25, pct=99%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper+allen_broadly_detectable, spec=-0.87, log2=9.02, pct=100%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Grm1[paper+allen_broadly_detectable, spec=-1.10, log2=7.39, pct=93%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-0.96, log2=10.19, pct=100%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-5.28, log2=1.04, pct=20%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-5.87, log2=6.56, pct=94%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Drd2[paper_only_allen_downgrade, spec=-1.32, log2=0.19, pct=3%; drugs: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect)]; Htr1a[paper_only_allen_downgrade, spec=-1.93, log2=1.39, pct=28%; drugs: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone]; Htr1b[paper_only_allen_downgrade, spec=-3.36, log2=0.05, pct=1%; drugs: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan]; Oprm1[paper_only_allen_downgrade, spec=-6.77, log2=0.19, pct=4%; drugs: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide]</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>allen_only_keep: Npy2r, Hcrtr1 | paper+broadly_detectable: Gabbr1, Gabbr2, Grm1, Grm5 | paper_only: Adcyap1r1(downgrade,spec=-5.28,log2=1.04); Cnr1(downgrade,spec=-5.87,log2=6.56); Drd2(downgrade,spec=-1.32,log2=0.19); Htr1a(downgrade,spec=-1.93,log2=1.39); Htr1b(downgrade,spec=-3.36,log2=0.05); Oprm1(downgrade,spec=-6.77,log2=0.19)</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>Npy2r | clinical/research: BIIE-0246 (research antagonist) | indication: food intake; anxiety (preclinical) || Hcrtr1 | clinical/research: SB-334867 (research selective antagonist) | indication: addiction; anxiety (preclinical) || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Drd2 | FDA: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect) | clinical/research: many | indication: schizophrenia; bipolar; Parkinson disease; hyperprolactinemia || Htr1a | FDA: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone | clinical/research: NLX-101 (depression) | indication: generalized anxiety; major depression || Htr1b | FDA: Sumatriptan; Rizatriptan; Zolmitriptan; Eletriptan; Naratriptan; Frovatriptan; Almotriptan | indication: migraine (acute attack) || Oprm1 | FDA: Morphine; Oxycodone; Hydrocodone; Methadone; Buprenorphine; Fentanyl; Tramadol; Naloxone (antag); Naltrexone (antag); Loperamide | clinical/research: PZM21 (biased agonist research) | indication: chronic pain; opioid use disorder; analgesia</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="110" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>DG granule cell</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>037 DG Glut</t>
         </is>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="8" t="n">
         <v>80255</v>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>C1ql2, Calb1, Dock10, Dsp, Prox1, Slc17a7</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Cnih3, Rgs14, Wfs1</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>Adcyap1r1, Cnr1, Drd2, Gabbr1, Gabbr2, Grm1, Grm5, Htr1a, Htr2c</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr"/>
-      <c r="I19" s="7" t="inlineStr">
-        <is>
-          <t>Adcyap1r1[paper_only_allen_downgrade, spec=-2.92, log2=3.40, pct=47%]; Cnr1[paper_only_allen_downgrade, spec=-11.77, log2=0.65, pct=10%]; Drd2[paper_only_allen_downgrade, spec=-1.50, log2=0.00, pct=0%]; Gabbr1[paper_only_allen_downgrade, spec=-2.51, log2=6.64, pct=82%]; Gabbr2[paper_only_allen_downgrade, spec=-2.13, log2=7.76, pct=89%]; Grm1[paper_only_allen_downgrade, spec=-0.06, log2=8.43, pct=93%]; Grm5[paper_only_allen_downgrade, spec=-0.98, log2=10.17, pct=99%]; Htr1a[paper_only_allen_downgrade, spec=-2.62, log2=0.71, pct=11%]; Htr2c[paper_only_allen_downgrade, spec=-11.79, log2=0.14, pct=2%]</t>
-        </is>
-      </c>
-      <c r="J19" s="7" t="inlineStr">
-        <is>
-          <t>paper_only: Adcyap1r1(downgrade,spec=-2.92,log2=3.40); Cnr1(downgrade,spec=-11.77,log2=0.65); Drd2(downgrade,spec=-1.50,log2=0.00); Gabbr1(downgrade,spec=-2.51,log2=6.64); Gabbr2(downgrade,spec=-2.13,log2=7.76); Grm1(downgrade,spec=-0.06,log2=8.43); Grm5(downgrade,spec=-0.98,log2=10.17); Htr1a(downgrade,spec=-2.62,log2=0.71); Htr2c(downgrade,spec=-11.79,log2=0.14)</t>
-        </is>
-      </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>no GPCR passes keep/validate thresholds; using expression fallback</t>
+      <c r="H19" s="8" t="inlineStr"/>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Grm1[paper+allen_broadly_detectable, spec=-0.06, log2=8.43, pct=93%; drugs: research_only_or_none]; Grm5[paper+allen_broadly_detectable, spec=-0.98, log2=10.17, pct=99%; drugs: research_only_or_none]; Adcyap1r1[paper_only_allen_downgrade, spec=-2.92, log2=3.40, pct=47%; drugs: research_only_or_none]; Cnr1[paper_only_allen_downgrade, spec=-11.77, log2=0.65, pct=10%; drugs: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action)]; Drd2[paper_only_allen_downgrade, spec=-1.50, log2=0.00, pct=0%; drugs: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect)]; Gabbr1[paper_only_allen_downgrade, spec=-2.51, log2=6.64, pct=82%; drugs: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem)]; Gabbr2[paper_only_allen_downgrade, spec=-2.13, log2=7.76, pct=89%; drugs: Baclofen (heterodimer with Gabbr1); Sodium oxybate]; Htr1a[paper_only_allen_downgrade, spec=-2.62, log2=0.71, pct=11%; drugs: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone]; Htr2c[paper_only_allen_downgrade, spec=-11.79, log2=0.14, pct=2%; drugs: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk)]</t>
+        </is>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>paper+broadly_detectable: Grm1, Grm5 | paper_only: Adcyap1r1(downgrade,spec=-2.92,log2=3.40); Cnr1(downgrade,spec=-11.77,log2=0.65); Drd2(downgrade,spec=-1.50,log2=0.00); Gabbr1(downgrade,spec=-2.51,log2=6.64); Gabbr2(downgrade,spec=-2.13,log2=7.76); Htr1a(downgrade,spec=-2.62,log2=0.71); Htr2c(downgrade,spec=-11.79,log2=0.14)</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>Grm1 | clinical/research: research mGluR1 negative allosteric modulators (CFMTI) | indication: chronic pain; cerebellar ataxia (preclinical) || Grm5 | clinical/research: Mavoglurant; Basimglurant; ADX-48621 (mostly failed Fragile X trials); Fenobam | indication: Fragile X syndrome (failed); anxiety; addiction (research) || Adcyap1r1 | clinical/research: Maxadilan; Atrasentan-related (research) | indication: migraine research || Cnr1 | FDA: Dronabinol (Marinol; THC); Nabilone; Cannabidiol (CBD; partial action) | clinical/research: Rimonabant (withdrawn obesity drug); JZP-150 | indication: appetite stimulation (cancer/AIDS); chemotherapy nausea; epilepsy (CBD) || Drd2 | FDA: Risperidone; Olanzapine; Aripiprazole; Quetiapine; Clozapine; Haloperidol; Paliperidone; Lurasidone; Bromocriptine; Cabergoline; Pramipexole; Ropinirole; Levodopa+Carbidopa (indirect) | clinical/research: many | indication: schizophrenia; bipolar; Parkinson disease; hyperprolactinemia || Gabbr1 | FDA: Baclofen (Lioresal); Arbaclofen Placarbil; Sodium oxybate (Xyrem) | clinical/research: Lesogaberan | indication: spasticity (multiple sclerosis; spinal cord injury); narcolepsy (Xyrem); alcohol use disorder (off-label) || Gabbr2 | FDA: Baclofen (heterodimer with Gabbr1); Sodium oxybate | clinical/research: (see Gabbr1) | indication: (see Gabbr1) || Htr1a | FDA: Buspirone; Vilazodone; Vortioxetine (partial); Tandospirone (Japan); Gepirone | clinical/research: NLX-101 (depression) | indication: generalized anxiety; major depression || Htr2c | FDA: Lorcaserin (Belviq) WITHDRAWN 2020 (cancer risk) | clinical/research: CT-7080; agomelatine (mixed) | indication: (historic obesity); current research for addiction</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>no cell-type-specific GPCR; relying on 2 broadly_expressed_detectable candidates</t>
         </is>
       </c>
     </row>

</xml_diff>